<commit_message>
&& - 86899520 от 12.03.2026 https://meshok.net/
</commit_message>
<xml_diff>
--- a/Collections/Russia/#Russia#Russian_Federation#Commemorative#[1999-present]#circulation_quality.xlsx
+++ b/Collections/Russia/#Russia#Russian_Federation#Commemorative#[1999-present]#circulation_quality.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\Russia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C69253C-C451-4253-87E3-ED388F1DCB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{250E2E82-2B1C-4CE4-8E91-40C34AF7C3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2633" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2623" uniqueCount="400">
   <si>
     <t>-</t>
   </si>
@@ -2319,14 +2319,15 @@
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="212">
+  <dxfs count="201">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -2335,95 +2336,6 @@
           <bgColor rgb="FF9BE5FF"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -4031,9 +3943,9 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="13" dataCellStyle="Гиперссылка"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="1" dataCellStyle="Гиперссылка"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -5092,7 +5004,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H3">
-    <cfRule type="containsText" dxfId="211" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="200" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5109,7 +5021,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5">
-    <cfRule type="containsText" dxfId="210" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="199" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G5))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5126,7 +5038,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="containsText" dxfId="209" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="198" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H5))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5143,7 +5055,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4">
-    <cfRule type="containsText" dxfId="208" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="197" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5160,7 +5072,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="containsText" dxfId="207" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="196" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5177,7 +5089,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G18:H18">
-    <cfRule type="containsText" dxfId="206" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="195" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5194,7 +5106,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:G17">
-    <cfRule type="containsText" dxfId="205" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="194" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G6))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5211,7 +5123,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H17">
-    <cfRule type="containsText" dxfId="204" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="193" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H6))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5228,7 +5140,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G19:G29">
-    <cfRule type="containsText" dxfId="203" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="192" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G19))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5245,7 +5157,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H19:H29">
-    <cfRule type="containsText" dxfId="202" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="191" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H19))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6378,7 +6290,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G4:H31">
-    <cfRule type="containsText" dxfId="201" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="190" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -6393,7 +6305,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="containsText" dxfId="200" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="189" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -6408,7 +6320,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3">
-    <cfRule type="containsText" dxfId="199" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="188" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6423,7 +6335,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G32:G39">
-    <cfRule type="containsText" dxfId="198" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="187" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -6438,7 +6350,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H32:H39">
-    <cfRule type="containsText" dxfId="197" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="186" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H32))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -8514,7 +8426,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G16:H65 G3:H8">
-    <cfRule type="containsText" dxfId="196" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="185" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -8529,7 +8441,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H66">
-    <cfRule type="containsText" dxfId="195" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="184" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H66))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -8544,7 +8456,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:G15">
-    <cfRule type="containsText" dxfId="194" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="183" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -8559,7 +8471,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:H15">
-    <cfRule type="containsText" dxfId="193" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="182" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -8574,7 +8486,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G67:G72">
-    <cfRule type="containsText" dxfId="192" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="181" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G67))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -8589,7 +8501,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H67:H72">
-    <cfRule type="containsText" dxfId="191" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="180" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H67))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -8604,7 +8516,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G66">
-    <cfRule type="containsText" dxfId="190" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="179" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G66))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14719,7 +14631,7 @@
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <conditionalFormatting sqref="G110:H167 G109 G4:H108">
-    <cfRule type="containsText" dxfId="189" priority="75" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="178" priority="75" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="76">
@@ -14734,7 +14646,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G168:H168">
-    <cfRule type="containsText" dxfId="188" priority="73" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="177" priority="73" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G168))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="74">
@@ -14749,7 +14661,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G169:H169">
-    <cfRule type="containsText" dxfId="187" priority="71" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="176" priority="71" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G169))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="72">
@@ -14764,7 +14676,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G170:H170">
-    <cfRule type="containsText" dxfId="186" priority="69" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="175" priority="69" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G170))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="70">
@@ -14779,7 +14691,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G171:H171">
-    <cfRule type="containsText" dxfId="185" priority="67" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="174" priority="67" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G171))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="68">
@@ -14794,7 +14706,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G172:H172">
-    <cfRule type="containsText" dxfId="184" priority="65" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="173" priority="65" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G172))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="66">
@@ -14809,7 +14721,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G173:H173">
-    <cfRule type="containsText" dxfId="183" priority="63" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="172" priority="63" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G173))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="64">
@@ -14824,7 +14736,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G174:H174">
-    <cfRule type="containsText" dxfId="182" priority="61" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="171" priority="61" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G174))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="62">
@@ -14839,7 +14751,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G175:H175">
-    <cfRule type="containsText" dxfId="181" priority="59" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="170" priority="59" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G175))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="60">
@@ -14854,7 +14766,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G176:H176">
-    <cfRule type="containsText" dxfId="180" priority="57" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="169" priority="57" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G176))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="58">
@@ -14869,7 +14781,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G177:H177">
-    <cfRule type="containsText" dxfId="179" priority="55" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="168" priority="55" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G177))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="56">
@@ -14884,7 +14796,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G178:H178">
-    <cfRule type="containsText" dxfId="178" priority="53" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="167" priority="53" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G178))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="54">
@@ -14899,7 +14811,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G179:H179">
-    <cfRule type="containsText" dxfId="177" priority="51" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="166" priority="51" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G179))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="52">
@@ -14914,7 +14826,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G180:H180">
-    <cfRule type="containsText" dxfId="176" priority="49" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="165" priority="49" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G180))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="50">
@@ -14929,7 +14841,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G181:H181">
-    <cfRule type="containsText" dxfId="175" priority="47" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="164" priority="47" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G181))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="48">
@@ -14944,7 +14856,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G182:H182">
-    <cfRule type="containsText" dxfId="174" priority="43" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="163" priority="43" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G182))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="44">
@@ -14959,7 +14871,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G183:H183">
-    <cfRule type="containsText" dxfId="173" priority="41" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="162" priority="41" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G183))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="42">
@@ -14974,7 +14886,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G184:H184">
-    <cfRule type="containsText" dxfId="172" priority="39" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="161" priority="39" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G184))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="40">
@@ -14989,7 +14901,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G186:H186">
-    <cfRule type="containsText" dxfId="171" priority="35" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="160" priority="35" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G186))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="36">
@@ -15004,7 +14916,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G187:H187">
-    <cfRule type="containsText" dxfId="170" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="159" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G187))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -15019,7 +14931,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G188:H188">
-    <cfRule type="containsText" dxfId="169" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="158" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G188))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -15034,7 +14946,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G185:H185">
-    <cfRule type="containsText" dxfId="168" priority="29" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="157" priority="29" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G185))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="30">
@@ -15049,7 +14961,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G189:H189">
-    <cfRule type="containsText" dxfId="167" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="156" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G189))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -15064,7 +14976,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G190:H190">
-    <cfRule type="containsText" dxfId="166" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="155" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G190))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -15079,7 +14991,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G191:H191">
-    <cfRule type="containsText" dxfId="165" priority="23" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="154" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G191))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -15094,7 +15006,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H109">
-    <cfRule type="containsText" dxfId="164" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="153" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H109))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15111,7 +15023,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:H3">
-    <cfRule type="containsText" dxfId="163" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="152" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -15126,7 +15038,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G192">
-    <cfRule type="containsText" dxfId="162" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="151" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G192))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -15141,7 +15053,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H192">
-    <cfRule type="containsText" dxfId="161" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="150" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H192))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -15156,7 +15068,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G193:H193 G195:H195 G197:H197">
-    <cfRule type="containsText" dxfId="160" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="149" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G193))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -15171,7 +15083,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G194:H194 G196:H196">
-    <cfRule type="containsText" dxfId="159" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="148" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G194))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -15186,7 +15098,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G198 G200">
-    <cfRule type="containsText" dxfId="158" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="147" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G198))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -15201,7 +15113,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H198 H200">
-    <cfRule type="containsText" dxfId="157" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="146" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H198))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -15216,7 +15128,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G199:H199 G201:H201">
-    <cfRule type="containsText" dxfId="156" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="145" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G199))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -15231,7 +15143,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G202:H202">
-    <cfRule type="containsText" dxfId="155" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="144" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G202))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -15246,7 +15158,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G203:H203">
-    <cfRule type="containsText" dxfId="154" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="143" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G203))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -15733,8 +15645,8 @@
       <c r="G16" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="H16" s="11" t="s">
-        <v>0</v>
+      <c r="H16" s="52">
+        <v>1</v>
       </c>
       <c r="I16" s="32"/>
     </row>
@@ -15788,8 +15700,8 @@
       <c r="G18" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="H18" s="11" t="s">
-        <v>0</v>
+      <c r="H18" s="52">
+        <v>1</v>
       </c>
       <c r="I18" s="32"/>
     </row>
@@ -15871,8 +15783,8 @@
       <c r="G21" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="H21" s="11" t="s">
-        <v>0</v>
+      <c r="H21" s="52">
+        <v>1</v>
       </c>
       <c r="I21" s="32"/>
     </row>
@@ -15982,8 +15894,8 @@
       <c r="G25" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="H25" s="11" t="s">
-        <v>0</v>
+      <c r="H25" s="52">
+        <v>1</v>
       </c>
       <c r="I25" s="32" t="str">
         <f t="shared" si="1"/>
@@ -16315,8 +16227,8 @@
       <c r="F37" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G37" s="11" t="s">
-        <v>0</v>
+      <c r="G37" s="52">
+        <v>1</v>
       </c>
       <c r="H37" s="11" t="s">
         <v>0</v>
@@ -16373,8 +16285,8 @@
       <c r="F39" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G39" s="11" t="s">
-        <v>0</v>
+      <c r="G39" s="52">
+        <v>1</v>
       </c>
       <c r="H39" s="11" t="s">
         <v>0</v>
@@ -16431,8 +16343,8 @@
       <c r="F41" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G41" s="11" t="s">
-        <v>0</v>
+      <c r="G41" s="52">
+        <v>1</v>
       </c>
       <c r="H41" s="11" t="s">
         <v>0</v>
@@ -16883,8 +16795,8 @@
       <c r="F57" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G57" s="11" t="s">
-        <v>0</v>
+      <c r="G57" s="52">
+        <v>1</v>
       </c>
       <c r="H57" s="11" t="s">
         <v>0</v>
@@ -17301,8 +17213,8 @@
       <c r="F72" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G72" s="11" t="s">
-        <v>0</v>
+      <c r="G72" s="52">
+        <v>1</v>
       </c>
       <c r="H72" s="11" t="s">
         <v>0</v>
@@ -17468,8 +17380,8 @@
       <c r="F78" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G78" s="11" t="s">
-        <v>0</v>
+      <c r="G78" s="52">
+        <v>1</v>
       </c>
       <c r="H78" s="11" t="s">
         <v>0</v>
@@ -17987,10 +17899,10 @@
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <conditionalFormatting sqref="G15:H15 G17:H17 G26:H26 G19:H20 G22:H24">
-    <cfRule type="containsText" dxfId="153" priority="428" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="142" priority="448" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G15))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="429">
+    <cfRule type="colorScale" priority="449">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18002,11 +17914,139 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="containsText" dxfId="152" priority="409" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="141" priority="429" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H26))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
+    <cfRule type="colorScale" priority="430">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28:H28">
+    <cfRule type="containsText" dxfId="140" priority="427" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G28))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="428">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H28">
+    <cfRule type="containsText" dxfId="139" priority="425" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H28))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H28">
+    <cfRule type="colorScale" priority="426">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="containsText" dxfId="138" priority="423" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="424">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="containsText" dxfId="137" priority="421" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="colorScale" priority="422">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G32:H32">
+    <cfRule type="containsText" dxfId="136" priority="415" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="416">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32">
+    <cfRule type="containsText" dxfId="135" priority="413" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H32))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32">
+    <cfRule type="colorScale" priority="414">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G34:H34 G38:H38">
+    <cfRule type="containsText" dxfId="134" priority="411" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G34))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="412">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H34 H38">
+    <cfRule type="containsText" dxfId="133" priority="409" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H34))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H38 H34">
     <cfRule type="colorScale" priority="410">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18018,9 +18058,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G28:H28">
-    <cfRule type="containsText" dxfId="151" priority="407" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G28))))</formula>
+  <conditionalFormatting sqref="G33:H33 G36:H36 G40:H40">
+    <cfRule type="containsText" dxfId="132" priority="407" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G33))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="408">
       <colorScale>
@@ -18033,12 +18073,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
-    <cfRule type="containsText" dxfId="150" priority="405" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H28))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
+  <conditionalFormatting sqref="H33 H36 H40">
+    <cfRule type="containsText" dxfId="131" priority="405" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36 H33 H40">
     <cfRule type="colorScale" priority="406">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18050,9 +18090,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="149" priority="403" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
+  <conditionalFormatting sqref="G42:H42">
+    <cfRule type="containsText" dxfId="130" priority="403" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G42))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="404">
       <colorScale>
@@ -18065,12 +18105,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="148" priority="401" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
+  <conditionalFormatting sqref="H42">
+    <cfRule type="containsText" dxfId="129" priority="401" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H42))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H42">
     <cfRule type="colorScale" priority="402">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18082,9 +18122,41 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G32:H32">
-    <cfRule type="containsText" dxfId="147" priority="395" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
+  <conditionalFormatting sqref="G43:H43">
+    <cfRule type="containsText" dxfId="128" priority="399" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G43))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="400">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H43">
+    <cfRule type="containsText" dxfId="127" priority="397" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H43))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H43">
+    <cfRule type="colorScale" priority="398">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G45:H45">
+    <cfRule type="containsText" dxfId="126" priority="395" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G45))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="396">
       <colorScale>
@@ -18097,12 +18169,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H32">
-    <cfRule type="containsText" dxfId="146" priority="393" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H32))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H32">
+  <conditionalFormatting sqref="H45">
+    <cfRule type="containsText" dxfId="125" priority="393" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H45))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45">
     <cfRule type="colorScale" priority="394">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18114,9 +18186,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G34:H34 G38:H38">
-    <cfRule type="containsText" dxfId="145" priority="391" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G34))))</formula>
+  <conditionalFormatting sqref="G47:H47 G49:H49 G51:H51 G53:H53 G55:H56 G54">
+    <cfRule type="containsText" dxfId="124" priority="391" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G47))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="392">
       <colorScale>
@@ -18129,12 +18201,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H34 H38">
-    <cfRule type="containsText" dxfId="144" priority="389" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H34))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H38 H34">
+  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
+    <cfRule type="containsText" dxfId="123" priority="389" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H47))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
     <cfRule type="colorScale" priority="390">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18146,9 +18218,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G33:H33 G36:H36 G40:H40">
-    <cfRule type="containsText" dxfId="143" priority="387" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G33))))</formula>
+  <conditionalFormatting sqref="G48:H48 G50:H50 G52:H52 H54">
+    <cfRule type="containsText" dxfId="122" priority="387" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G48))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="388">
       <colorScale>
@@ -18161,12 +18233,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H33 H36 H40">
-    <cfRule type="containsText" dxfId="142" priority="385" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H36 H33 H40">
+  <conditionalFormatting sqref="H48 H50 H52 H54">
+    <cfRule type="containsText" dxfId="121" priority="385" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H48))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H50 H48 H52 H54">
     <cfRule type="colorScale" priority="386">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18178,11 +18250,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G42:H42">
-    <cfRule type="containsText" dxfId="141" priority="383" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G42))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="384">
+  <conditionalFormatting sqref="G61:H61 G63:H63 G65:H65 G67:H67 G69:H69">
+    <cfRule type="containsText" dxfId="120" priority="363" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G61))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="364">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18193,13 +18265,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H42">
-    <cfRule type="containsText" dxfId="140" priority="381" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H42))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H42">
-    <cfRule type="colorScale" priority="382">
+  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
+    <cfRule type="containsText" dxfId="119" priority="361" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H61))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
+    <cfRule type="colorScale" priority="362">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18210,11 +18282,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G43:H43">
-    <cfRule type="containsText" dxfId="139" priority="379" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G43))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="380">
+  <conditionalFormatting sqref="G60:H60 G62:H62 G64:H64 G66:H66 G68:H68 G70:H70 G73:H73">
+    <cfRule type="containsText" dxfId="118" priority="359" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G60))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="360">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18225,13 +18297,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H43">
-    <cfRule type="containsText" dxfId="138" priority="377" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H43))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H43">
-    <cfRule type="colorScale" priority="378">
+  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
+    <cfRule type="containsText" dxfId="117" priority="357" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H60))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
+    <cfRule type="colorScale" priority="358">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18242,11 +18314,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G45:H45">
-    <cfRule type="containsText" dxfId="137" priority="375" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G45))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="376">
+  <conditionalFormatting sqref="G58:H58">
+    <cfRule type="containsText" dxfId="116" priority="355" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G58))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="356">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18257,13 +18329,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H45">
-    <cfRule type="containsText" dxfId="136" priority="373" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H45))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45">
-    <cfRule type="colorScale" priority="374">
+  <conditionalFormatting sqref="H58">
+    <cfRule type="containsText" dxfId="115" priority="353" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H58))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H58">
+    <cfRule type="colorScale" priority="354">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18274,11 +18346,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G47:H47 G49:H49 G51:H51 G53:H53 G55:H56 G54">
-    <cfRule type="containsText" dxfId="135" priority="371" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G47))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="372">
+  <conditionalFormatting sqref="G71:H71">
+    <cfRule type="containsText" dxfId="114" priority="351" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G71))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="352">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18289,13 +18361,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
-    <cfRule type="containsText" dxfId="134" priority="369" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H47))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
-    <cfRule type="colorScale" priority="370">
+  <conditionalFormatting sqref="H71">
+    <cfRule type="containsText" dxfId="113" priority="349" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H71))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H71">
+    <cfRule type="colorScale" priority="350">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18306,105 +18378,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G48:H48 G50:H50 G52:H52 H54">
-    <cfRule type="containsText" dxfId="133" priority="367" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G48))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="368">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H48 H50 H52 H54">
-    <cfRule type="containsText" dxfId="132" priority="365" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H48))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H50 H48 H52 H54">
-    <cfRule type="colorScale" priority="366">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G61:H61 G63:H63 G65:H65 G67:H67 G69:H69">
-    <cfRule type="containsText" dxfId="131" priority="343" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G61))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="344">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
-    <cfRule type="containsText" dxfId="130" priority="341" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H61))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
-    <cfRule type="colorScale" priority="342">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G60:H60 G62:H62 G64:H64 G66:H66 G68:H68 G70:H70 G73:H73">
-    <cfRule type="containsText" dxfId="129" priority="339" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G60))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="340">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
-    <cfRule type="containsText" dxfId="128" priority="337" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H60))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
-    <cfRule type="colorScale" priority="338">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G58:H58">
-    <cfRule type="containsText" dxfId="127" priority="335" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G58))))</formula>
+  <conditionalFormatting sqref="G22">
+    <cfRule type="containsText" dxfId="112" priority="335" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G22))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="336">
       <colorScale>
@@ -18417,12 +18393,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H58">
-    <cfRule type="containsText" dxfId="126" priority="333" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H58))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H58">
+  <conditionalFormatting sqref="H22">
+    <cfRule type="containsText" dxfId="111" priority="333" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H22))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="334">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18434,9 +18408,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G71:H71">
-    <cfRule type="containsText" dxfId="125" priority="331" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G71))))</formula>
+  <conditionalFormatting sqref="G25">
+    <cfRule type="containsText" dxfId="110" priority="331" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G25))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="332">
       <colorScale>
@@ -18449,13 +18423,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H71">
-    <cfRule type="containsText" dxfId="124" priority="329" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H71))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H71">
-    <cfRule type="colorScale" priority="330">
+  <conditionalFormatting sqref="G27:H27">
+    <cfRule type="containsText" dxfId="109" priority="323" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="324">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18466,11 +18438,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G22">
-    <cfRule type="containsText" dxfId="123" priority="315" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G22))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="316">
+  <conditionalFormatting sqref="H27">
+    <cfRule type="containsText" dxfId="108" priority="321" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H27))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="colorScale" priority="322">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18481,11 +18455,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H22">
-    <cfRule type="containsText" dxfId="122" priority="313" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H22))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="314">
+  <conditionalFormatting sqref="G75:H75">
+    <cfRule type="containsText" dxfId="107" priority="271" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G75))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="272">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18496,11 +18470,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G25">
-    <cfRule type="containsText" dxfId="121" priority="311" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G25))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="312">
+  <conditionalFormatting sqref="H75">
+    <cfRule type="containsText" dxfId="106" priority="269" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H75))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H75">
+    <cfRule type="colorScale" priority="270">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18511,11 +18487,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G27:H27">
-    <cfRule type="containsText" dxfId="120" priority="303" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="304">
+  <conditionalFormatting sqref="G77:H77">
+    <cfRule type="containsText" dxfId="105" priority="263" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G77))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="264">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18526,13 +18502,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="containsText" dxfId="119" priority="301" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H27))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="colorScale" priority="302">
+  <conditionalFormatting sqref="H77">
+    <cfRule type="containsText" dxfId="104" priority="261" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H77))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H77">
+    <cfRule type="colorScale" priority="262">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18543,9 +18519,41 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G75:H75">
-    <cfRule type="containsText" dxfId="118" priority="251" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G75))))</formula>
+  <conditionalFormatting sqref="G79:H79">
+    <cfRule type="containsText" dxfId="103" priority="255" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G79))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="256">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H79">
+    <cfRule type="containsText" dxfId="102" priority="253" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H79))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H79">
+    <cfRule type="colorScale" priority="254">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G81:H81">
+    <cfRule type="containsText" dxfId="101" priority="251" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G81))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="252">
       <colorScale>
@@ -18558,12 +18566,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H75">
-    <cfRule type="containsText" dxfId="117" priority="249" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H75))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H75">
+  <conditionalFormatting sqref="H81">
+    <cfRule type="containsText" dxfId="100" priority="249" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H81))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H81">
     <cfRule type="colorScale" priority="250">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18575,9 +18583,41 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G77:H77">
-    <cfRule type="containsText" dxfId="116" priority="243" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G77))))</formula>
+  <conditionalFormatting sqref="G83:H83">
+    <cfRule type="containsText" dxfId="99" priority="247" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G83))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="248">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H83">
+    <cfRule type="containsText" dxfId="98" priority="245" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H83))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H83">
+    <cfRule type="colorScale" priority="246">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G85:H85">
+    <cfRule type="containsText" dxfId="97" priority="243" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G85))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="244">
       <colorScale>
@@ -18590,12 +18630,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H77">
-    <cfRule type="containsText" dxfId="115" priority="241" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H77))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H77">
+  <conditionalFormatting sqref="H85">
+    <cfRule type="containsText" dxfId="96" priority="241" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H85))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H85">
     <cfRule type="colorScale" priority="242">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18607,106 +18647,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G79:H79">
-    <cfRule type="containsText" dxfId="114" priority="235" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G79))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="236">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H79">
-    <cfRule type="containsText" dxfId="113" priority="233" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H79))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H79">
-    <cfRule type="colorScale" priority="234">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G81:H81">
-    <cfRule type="containsText" dxfId="112" priority="231" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G81))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="232">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="containsText" dxfId="111" priority="229" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H81))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="colorScale" priority="230">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G83:H83">
-    <cfRule type="containsText" dxfId="110" priority="227" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G83))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="228">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H83">
-    <cfRule type="containsText" dxfId="109" priority="225" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H83))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H83">
-    <cfRule type="colorScale" priority="226">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G85:H85">
-    <cfRule type="containsText" dxfId="108" priority="223" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G85))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="G27">
+    <cfRule type="containsText" dxfId="95" priority="223" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27">
     <cfRule type="colorScale" priority="224">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18718,12 +18664,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H85">
-    <cfRule type="containsText" dxfId="107" priority="221" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H85))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H85">
+  <conditionalFormatting sqref="G29:H29">
+    <cfRule type="containsText" dxfId="94" priority="221" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="222">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18735,12 +18679,142 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
-    <cfRule type="containsText" dxfId="106" priority="203" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
+  <conditionalFormatting sqref="H29">
+    <cfRule type="containsText" dxfId="93" priority="219" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29">
+    <cfRule type="colorScale" priority="220">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="containsText" dxfId="92" priority="217" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="colorScale" priority="218">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35:H35">
+    <cfRule type="containsText" dxfId="91" priority="215" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="216">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="containsText" dxfId="90" priority="213" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="colorScale" priority="214">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35">
+    <cfRule type="containsText" dxfId="89" priority="211" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35">
+    <cfRule type="colorScale" priority="212">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44:H44">
+    <cfRule type="containsText" dxfId="88" priority="209" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="210">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H44">
+    <cfRule type="containsText" dxfId="87" priority="207" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H44))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H44">
+    <cfRule type="colorScale" priority="208">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44">
+    <cfRule type="containsText" dxfId="86" priority="205" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44">
+    <cfRule type="colorScale" priority="206">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H46">
+    <cfRule type="containsText" dxfId="85" priority="203" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="204">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18752,10 +18826,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G29:H29">
-    <cfRule type="containsText" dxfId="105" priority="201" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H46">
+    <cfRule type="containsText" dxfId="84" priority="201" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H46">
     <cfRule type="colorScale" priority="202">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18767,29 +18843,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
-    <cfRule type="containsText" dxfId="104" priority="199" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
-    <cfRule type="colorScale" priority="200">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
-    <cfRule type="containsText" dxfId="103" priority="197" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
+  <conditionalFormatting sqref="H59">
+    <cfRule type="containsText" dxfId="83" priority="197" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="198">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18801,10 +18858,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G35:H35">
-    <cfRule type="containsText" dxfId="102" priority="195" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H59">
+    <cfRule type="containsText" dxfId="82" priority="195" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H59">
     <cfRule type="colorScale" priority="196">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18816,29 +18875,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H35">
-    <cfRule type="containsText" dxfId="101" priority="193" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H35">
-    <cfRule type="colorScale" priority="194">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
-    <cfRule type="containsText" dxfId="100" priority="191" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
+  <conditionalFormatting sqref="H57">
+    <cfRule type="containsText" dxfId="81" priority="191" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="192">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18850,10 +18890,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G44:H44">
-    <cfRule type="containsText" dxfId="99" priority="189" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H57">
+    <cfRule type="containsText" dxfId="80" priority="189" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H57">
     <cfRule type="colorScale" priority="190">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18865,29 +18907,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H44">
-    <cfRule type="containsText" dxfId="98" priority="187" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H44))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H44">
-    <cfRule type="colorScale" priority="188">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G44">
-    <cfRule type="containsText" dxfId="97" priority="185" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G44">
+  <conditionalFormatting sqref="H80">
+    <cfRule type="containsText" dxfId="79" priority="185" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="186">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18899,10 +18922,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
-    <cfRule type="containsText" dxfId="96" priority="183" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H80">
+    <cfRule type="containsText" dxfId="78" priority="183" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H80">
     <cfRule type="colorScale" priority="184">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18914,13 +18939,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
-    <cfRule type="containsText" dxfId="95" priority="181" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
-    <cfRule type="colorScale" priority="182">
+  <conditionalFormatting sqref="H78">
+    <cfRule type="containsText" dxfId="77" priority="179" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="180">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18931,10 +18954,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H59">
-    <cfRule type="containsText" dxfId="93" priority="177" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H78">
+    <cfRule type="containsText" dxfId="76" priority="177" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H78">
     <cfRule type="colorScale" priority="178">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18946,13 +18971,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H59">
-    <cfRule type="containsText" dxfId="92" priority="175" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H59">
-    <cfRule type="colorScale" priority="176">
+  <conditionalFormatting sqref="H76">
+    <cfRule type="containsText" dxfId="75" priority="173" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="174">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18963,10 +18986,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G57:H57">
-    <cfRule type="containsText" dxfId="90" priority="171" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G57))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H76">
+    <cfRule type="containsText" dxfId="74" priority="171" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H76">
     <cfRule type="colorScale" priority="172">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18978,29 +19003,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H57">
-    <cfRule type="containsText" dxfId="89" priority="169" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H57">
-    <cfRule type="colorScale" priority="170">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57">
-    <cfRule type="containsText" dxfId="88" priority="167" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G57))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57">
+  <conditionalFormatting sqref="H74">
+    <cfRule type="containsText" dxfId="73" priority="167" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="168">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19012,10 +19018,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H80">
-    <cfRule type="containsText" dxfId="87" priority="165" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H74">
+    <cfRule type="containsText" dxfId="72" priority="165" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H74">
     <cfRule type="colorScale" priority="166">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19027,13 +19035,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H80">
-    <cfRule type="containsText" dxfId="86" priority="163" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H80">
-    <cfRule type="colorScale" priority="164">
+  <conditionalFormatting sqref="H72">
+    <cfRule type="containsText" dxfId="71" priority="161" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="162">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19044,10 +19050,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G78:H78">
-    <cfRule type="containsText" dxfId="84" priority="159" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G78))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H72">
+    <cfRule type="containsText" dxfId="70" priority="159" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H72">
     <cfRule type="colorScale" priority="160">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19059,29 +19067,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H78">
-    <cfRule type="containsText" dxfId="83" priority="157" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H78">
-    <cfRule type="colorScale" priority="158">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G78">
-    <cfRule type="containsText" dxfId="82" priority="155" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G78))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G78">
+  <conditionalFormatting sqref="H82">
+    <cfRule type="containsText" dxfId="69" priority="155" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="156">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19093,10 +19082,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H76">
-    <cfRule type="containsText" dxfId="81" priority="153" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H82">
+    <cfRule type="containsText" dxfId="68" priority="153" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H82">
     <cfRule type="colorScale" priority="154">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19108,13 +19099,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H76">
-    <cfRule type="containsText" dxfId="80" priority="151" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H76">
-    <cfRule type="colorScale" priority="152">
+  <conditionalFormatting sqref="H86">
+    <cfRule type="containsText" dxfId="67" priority="149" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="150">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19125,10 +19114,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H74">
-    <cfRule type="containsText" dxfId="78" priority="147" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H86">
+    <cfRule type="containsText" dxfId="66" priority="147" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H86">
     <cfRule type="colorScale" priority="148">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19140,13 +19131,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H74">
-    <cfRule type="containsText" dxfId="77" priority="145" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H74">
-    <cfRule type="colorScale" priority="146">
+  <conditionalFormatting sqref="H84">
+    <cfRule type="containsText" dxfId="65" priority="143" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="144">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19157,10 +19146,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G72:H72">
-    <cfRule type="containsText" dxfId="75" priority="141" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G72))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H84">
+    <cfRule type="containsText" dxfId="64" priority="141" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H84">
     <cfRule type="colorScale" priority="142">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19172,29 +19163,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H72">
-    <cfRule type="containsText" dxfId="74" priority="139" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H72">
-    <cfRule type="colorScale" priority="140">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G72">
-    <cfRule type="containsText" dxfId="73" priority="137" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G72))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G72">
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="63" priority="137" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="138">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19206,10 +19178,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H82">
-    <cfRule type="containsText" dxfId="72" priority="135" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="62" priority="135" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
     <cfRule type="colorScale" priority="136">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19221,13 +19195,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H82">
-    <cfRule type="containsText" dxfId="71" priority="133" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H82">
-    <cfRule type="colorScale" priority="134">
+  <conditionalFormatting sqref="H41">
+    <cfRule type="containsText" dxfId="61" priority="131" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="132">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19238,10 +19210,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
-    <cfRule type="containsText" dxfId="69" priority="129" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H41">
+    <cfRule type="containsText" dxfId="60" priority="129" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H41">
     <cfRule type="colorScale" priority="130">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19253,13 +19227,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
-    <cfRule type="containsText" dxfId="68" priority="127" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
-    <cfRule type="colorScale" priority="128">
+  <conditionalFormatting sqref="H39">
+    <cfRule type="containsText" dxfId="59" priority="125" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="126">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19270,10 +19242,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H84">
-    <cfRule type="containsText" dxfId="66" priority="123" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H39">
+    <cfRule type="containsText" dxfId="58" priority="123" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H39">
     <cfRule type="colorScale" priority="124">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19285,26 +19259,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H84">
-    <cfRule type="containsText" dxfId="65" priority="121" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H84">
-    <cfRule type="colorScale" priority="122">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G37:H37">
-    <cfRule type="containsText" dxfId="63" priority="117" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G37))))</formula>
+  <conditionalFormatting sqref="G21">
+    <cfRule type="containsText" dxfId="57" priority="117" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G21))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="118">
       <colorScale>
@@ -19317,29 +19274,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
-    <cfRule type="containsText" dxfId="62" priority="115" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
-    <cfRule type="colorScale" priority="116">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G37">
-    <cfRule type="containsText" dxfId="61" priority="113" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G37))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G37">
+  <conditionalFormatting sqref="G18">
+    <cfRule type="containsText" dxfId="56" priority="113" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="114">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19351,27 +19289,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G41:H41">
-    <cfRule type="containsText" dxfId="60" priority="111" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G41))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="112">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H41">
-    <cfRule type="containsText" dxfId="59" priority="109" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H41">
+  <conditionalFormatting sqref="G16">
+    <cfRule type="containsText" dxfId="55" priority="109" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G16))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="110">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19383,44 +19304,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G41">
-    <cfRule type="containsText" dxfId="58" priority="107" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G41))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G41">
-    <cfRule type="colorScale" priority="108">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G39:H39">
-    <cfRule type="containsText" dxfId="57" priority="105" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G39))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="106">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H39">
-    <cfRule type="containsText" dxfId="56" priority="103" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H39">
+  <conditionalFormatting sqref="H31">
+    <cfRule type="containsText" dxfId="54" priority="103" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="104">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19432,12 +19319,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G39">
-    <cfRule type="containsText" dxfId="55" priority="101" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G39))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G39">
+  <conditionalFormatting sqref="H31">
+    <cfRule type="containsText" dxfId="53" priority="101" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H31">
     <cfRule type="colorScale" priority="102">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19449,24 +19336,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H25">
-    <cfRule type="containsText" dxfId="54" priority="99" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H25))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="100">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G21">
-    <cfRule type="containsText" dxfId="53" priority="97" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G21))))</formula>
+  <conditionalFormatting sqref="G3:H8">
+    <cfRule type="containsText" dxfId="52" priority="97" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="98">
       <colorScale>
@@ -19479,9 +19351,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
-    <cfRule type="containsText" dxfId="52" priority="95" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H21))))</formula>
+  <conditionalFormatting sqref="G9:G14">
+    <cfRule type="containsText" dxfId="51" priority="95" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="96">
       <colorScale>
@@ -19494,9 +19366,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G18">
-    <cfRule type="containsText" dxfId="51" priority="93" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
+  <conditionalFormatting sqref="H9:H14">
+    <cfRule type="containsText" dxfId="50" priority="93" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="94">
       <colorScale>
@@ -19509,9 +19381,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H18">
-    <cfRule type="containsText" dxfId="50" priority="91" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H18))))</formula>
+  <conditionalFormatting sqref="G87:H87">
+    <cfRule type="containsText" dxfId="49" priority="91" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G87))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="92">
       <colorScale>
@@ -19524,10 +19396,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16">
-    <cfRule type="containsText" dxfId="49" priority="89" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G16))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H87">
+    <cfRule type="containsText" dxfId="48" priority="89" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H87))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H87">
     <cfRule type="colorScale" priority="90">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19539,9 +19413,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="48" priority="87" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
+  <conditionalFormatting sqref="H88">
+    <cfRule type="containsText" dxfId="47" priority="87" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="88">
       <colorScale>
@@ -19554,11 +19428,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
-    <cfRule type="containsText" dxfId="47" priority="83" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="84">
+  <conditionalFormatting sqref="H88">
+    <cfRule type="containsText" dxfId="46" priority="85" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H88">
+    <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19569,12 +19445,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
-    <cfRule type="containsText" dxfId="46" priority="81" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
+  <conditionalFormatting sqref="G31">
+    <cfRule type="containsText" dxfId="45" priority="81" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G31))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="82">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19586,10 +19460,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:H8">
-    <cfRule type="containsText" dxfId="45" priority="77" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="G89:H89">
+    <cfRule type="containsText" dxfId="44" priority="79" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G89))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="80">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H89">
+    <cfRule type="containsText" dxfId="43" priority="77" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H89))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H89">
     <cfRule type="colorScale" priority="78">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19601,9 +19492,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:G14">
-    <cfRule type="containsText" dxfId="44" priority="75" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G9))))</formula>
+  <conditionalFormatting sqref="H90">
+    <cfRule type="containsText" dxfId="42" priority="75" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="76">
       <colorScale>
@@ -19616,10 +19507,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H14">
-    <cfRule type="containsText" dxfId="43" priority="73" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H90">
+    <cfRule type="containsText" dxfId="41" priority="73" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H90">
     <cfRule type="colorScale" priority="74">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19631,27 +19524,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G87:H87">
-    <cfRule type="containsText" dxfId="42" priority="71" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G87))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="72">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H87">
-    <cfRule type="containsText" dxfId="41" priority="69" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H87))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H87">
+  <conditionalFormatting sqref="H91:H94">
+    <cfRule type="containsText" dxfId="40" priority="69" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="70">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19663,10 +19539,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="40" priority="67" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H91:H94">
+    <cfRule type="containsText" dxfId="39" priority="67" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H91:H94">
     <cfRule type="colorScale" priority="68">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19678,12 +19556,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="39" priority="65" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
+  <conditionalFormatting sqref="H95">
+    <cfRule type="containsText" dxfId="38" priority="65" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="66">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19695,11 +19571,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G31">
-    <cfRule type="containsText" dxfId="37" priority="61" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G31))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="62">
+  <conditionalFormatting sqref="H95">
+    <cfRule type="containsText" dxfId="37" priority="63" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H95">
+    <cfRule type="colorScale" priority="64">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19710,10 +19588,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G89:H89">
+  <conditionalFormatting sqref="G30">
     <cfRule type="containsText" dxfId="36" priority="59" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G89))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G30))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30">
     <cfRule type="colorScale" priority="60">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19725,12 +19605,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H89">
+  <conditionalFormatting sqref="G91">
     <cfRule type="containsText" dxfId="35" priority="57" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H89))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H89">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G91))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G91">
     <cfRule type="colorScale" priority="58">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19742,10 +19622,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H90">
+  <conditionalFormatting sqref="G92">
     <cfRule type="containsText" dxfId="34" priority="55" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G92))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G92">
     <cfRule type="colorScale" priority="56">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19757,12 +19639,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H90">
+  <conditionalFormatting sqref="G93">
     <cfRule type="containsText" dxfId="33" priority="53" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H90">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G93))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G93">
     <cfRule type="colorScale" priority="54">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19774,10 +19656,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H91:H94">
+  <conditionalFormatting sqref="G94">
     <cfRule type="containsText" dxfId="32" priority="49" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G94))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G94">
     <cfRule type="colorScale" priority="50">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19789,12 +19673,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H91:H94">
+  <conditionalFormatting sqref="G95">
     <cfRule type="containsText" dxfId="31" priority="47" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H91:H94">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G95))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G95">
     <cfRule type="colorScale" priority="48">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19806,10 +19690,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H95">
+  <conditionalFormatting sqref="G90">
     <cfRule type="containsText" dxfId="30" priority="45" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G90))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G90">
     <cfRule type="colorScale" priority="46">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19821,13 +19707,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H95">
-    <cfRule type="containsText" dxfId="29" priority="43" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H95">
-    <cfRule type="colorScale" priority="44">
+  <conditionalFormatting sqref="G59">
+    <cfRule type="containsText" dxfId="29" priority="41" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G59))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G59">
+    <cfRule type="colorScale" priority="42">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19838,12 +19724,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
+  <conditionalFormatting sqref="G76">
     <cfRule type="containsText" dxfId="28" priority="39" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G30))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G76))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G76">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19855,29 +19741,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G91">
-    <cfRule type="containsText" dxfId="27" priority="37" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G91))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G91">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G92">
-    <cfRule type="containsText" dxfId="26" priority="35" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G92))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G92">
+  <conditionalFormatting sqref="G80">
+    <cfRule type="containsText" dxfId="27" priority="35" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G80))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G80">
     <cfRule type="colorScale" priority="36">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19889,12 +19758,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G93">
-    <cfRule type="containsText" dxfId="25" priority="33" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G93))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G93">
+  <conditionalFormatting sqref="G82">
+    <cfRule type="containsText" dxfId="26" priority="33" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G82))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G82">
     <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19906,12 +19775,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G94">
+  <conditionalFormatting sqref="G84">
+    <cfRule type="containsText" dxfId="25" priority="31" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G84))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G84">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G88">
     <cfRule type="containsText" dxfId="24" priority="29" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G94))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G94">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G88))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G88">
     <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19923,12 +19809,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G95">
+  <conditionalFormatting sqref="G86">
     <cfRule type="containsText" dxfId="23" priority="27" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G95))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G95">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G86))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G86">
     <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19940,12 +19826,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G90">
+  <conditionalFormatting sqref="G46">
     <cfRule type="containsText" dxfId="22" priority="25" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G90))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G90">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19957,12 +19841,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G59">
-    <cfRule type="containsText" dxfId="10" priority="21" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G59))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G59">
+  <conditionalFormatting sqref="G46">
+    <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G46">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G74">
+    <cfRule type="containsText" dxfId="20" priority="21" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G74))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G74">
     <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19974,12 +19875,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G76">
-    <cfRule type="containsText" dxfId="9" priority="19" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G76))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G76">
+  <conditionalFormatting sqref="G57">
+    <cfRule type="containsText" dxfId="19" priority="19" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G57))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G57">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19992,7 +19893,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G78">
-    <cfRule type="containsText" dxfId="8" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="18" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G78))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20008,12 +19909,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G80">
-    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G80))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G80">
+  <conditionalFormatting sqref="H16">
+    <cfRule type="containsText" dxfId="17" priority="15" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20025,12 +19926,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G82">
-    <cfRule type="containsText" dxfId="6" priority="13" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G82))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G82">
+  <conditionalFormatting sqref="H18">
+    <cfRule type="containsText" dxfId="16" priority="13" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H18))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20042,12 +19943,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G84">
-    <cfRule type="containsText" dxfId="5" priority="11" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G84))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G84">
+  <conditionalFormatting sqref="H21">
+    <cfRule type="containsText" dxfId="15" priority="11" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H21))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H21">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20059,12 +19960,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G88">
-    <cfRule type="containsText" dxfId="4" priority="9" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G88))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G88">
+  <conditionalFormatting sqref="H25">
+    <cfRule type="containsText" dxfId="14" priority="9" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H25))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20076,12 +19977,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G86">
-    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G86))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G86">
+  <conditionalFormatting sqref="G41">
+    <cfRule type="containsText" dxfId="13" priority="7" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G41))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G41">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20093,10 +19994,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
-    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="G39">
+    <cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G39))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G39">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20108,12 +20011,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
+  <conditionalFormatting sqref="G37">
+    <cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20125,12 +20028,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G74">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G74))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G74">
+  <conditionalFormatting sqref="G72">
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G72))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G72">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -21046,7 +20949,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H28">
-    <cfRule type="containsText" dxfId="21" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="9" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -21061,7 +20964,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H29">
-    <cfRule type="containsText" dxfId="20" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="8" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -21076,7 +20979,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H29">
-    <cfRule type="containsText" dxfId="19" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="7" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21093,7 +20996,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G29">
-    <cfRule type="containsText" dxfId="18" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="6" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21110,7 +21013,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="17" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="5" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -21125,7 +21028,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="16" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21142,7 +21045,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30">
-    <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G30))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">

</xml_diff>

<commit_message>
&&& - 86899572 от 12.03.2026 https://meshok.net/
</commit_message>
<xml_diff>
--- a/Collections/Russia/#Russia#Russian_Federation#Commemorative#[1999-present]#circulation_quality.xlsx
+++ b/Collections/Russia/#Russia#Russian_Federation#Commemorative#[1999-present]#circulation_quality.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\Russia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{250E2E82-2B1C-4CE4-8E91-40C34AF7C3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F2A2BF-A369-4D0F-992D-66862191D5AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2623" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2618" uniqueCount="400">
   <si>
     <t>-</t>
   </si>
@@ -2319,7 +2319,47 @@
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="201">
+  <dxfs count="206">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -3943,9 +3983,9 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="1" dataCellStyle="Гиперссылка"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="6" dataCellStyle="Гиперссылка"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -5004,7 +5044,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H3">
-    <cfRule type="containsText" dxfId="200" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="205" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5021,7 +5061,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5">
-    <cfRule type="containsText" dxfId="199" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="204" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G5))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5038,7 +5078,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="containsText" dxfId="198" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="203" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H5))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5055,7 +5095,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4">
-    <cfRule type="containsText" dxfId="197" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="202" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5072,7 +5112,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4">
-    <cfRule type="containsText" dxfId="196" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="201" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5089,7 +5129,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G18:H18">
-    <cfRule type="containsText" dxfId="195" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="200" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5106,7 +5146,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:G17">
-    <cfRule type="containsText" dxfId="194" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="199" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G6))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5123,7 +5163,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H17">
-    <cfRule type="containsText" dxfId="193" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="198" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H6))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5140,7 +5180,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G19:G29">
-    <cfRule type="containsText" dxfId="192" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="197" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G19))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5157,7 +5197,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H19:H29">
-    <cfRule type="containsText" dxfId="191" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="196" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H19))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6290,7 +6330,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G4:H31">
-    <cfRule type="containsText" dxfId="190" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="195" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -6305,7 +6345,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="containsText" dxfId="189" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="194" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -6320,7 +6360,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3">
-    <cfRule type="containsText" dxfId="188" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="193" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6335,7 +6375,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G32:G39">
-    <cfRule type="containsText" dxfId="187" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="192" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -6350,7 +6390,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H32:H39">
-    <cfRule type="containsText" dxfId="186" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="191" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H32))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -8426,7 +8466,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G16:H65 G3:H8">
-    <cfRule type="containsText" dxfId="185" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="190" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -8441,7 +8481,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H66">
-    <cfRule type="containsText" dxfId="184" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="189" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H66))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -8456,7 +8496,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:G15">
-    <cfRule type="containsText" dxfId="183" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="188" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -8471,7 +8511,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:H15">
-    <cfRule type="containsText" dxfId="182" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="187" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -8486,7 +8526,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G67:G72">
-    <cfRule type="containsText" dxfId="181" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="186" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G67))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -8501,7 +8541,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H67:H72">
-    <cfRule type="containsText" dxfId="180" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="185" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H67))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -8516,7 +8556,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G66">
-    <cfRule type="containsText" dxfId="179" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="184" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G66))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14631,7 +14671,7 @@
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <conditionalFormatting sqref="G110:H167 G109 G4:H108">
-    <cfRule type="containsText" dxfId="178" priority="75" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="183" priority="75" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G4))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="76">
@@ -14646,7 +14686,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G168:H168">
-    <cfRule type="containsText" dxfId="177" priority="73" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="182" priority="73" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G168))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="74">
@@ -14661,7 +14701,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G169:H169">
-    <cfRule type="containsText" dxfId="176" priority="71" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="181" priority="71" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G169))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="72">
@@ -14676,7 +14716,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G170:H170">
-    <cfRule type="containsText" dxfId="175" priority="69" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="180" priority="69" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G170))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="70">
@@ -14691,7 +14731,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G171:H171">
-    <cfRule type="containsText" dxfId="174" priority="67" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="179" priority="67" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G171))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="68">
@@ -14706,7 +14746,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G172:H172">
-    <cfRule type="containsText" dxfId="173" priority="65" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="178" priority="65" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G172))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="66">
@@ -14721,7 +14761,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G173:H173">
-    <cfRule type="containsText" dxfId="172" priority="63" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="177" priority="63" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G173))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="64">
@@ -14736,7 +14776,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G174:H174">
-    <cfRule type="containsText" dxfId="171" priority="61" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="176" priority="61" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G174))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="62">
@@ -14751,7 +14791,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G175:H175">
-    <cfRule type="containsText" dxfId="170" priority="59" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="175" priority="59" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G175))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="60">
@@ -14766,7 +14806,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G176:H176">
-    <cfRule type="containsText" dxfId="169" priority="57" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="174" priority="57" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G176))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="58">
@@ -14781,7 +14821,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G177:H177">
-    <cfRule type="containsText" dxfId="168" priority="55" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="173" priority="55" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G177))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="56">
@@ -14796,7 +14836,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G178:H178">
-    <cfRule type="containsText" dxfId="167" priority="53" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="172" priority="53" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G178))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="54">
@@ -14811,7 +14851,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G179:H179">
-    <cfRule type="containsText" dxfId="166" priority="51" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="171" priority="51" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G179))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="52">
@@ -14826,7 +14866,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G180:H180">
-    <cfRule type="containsText" dxfId="165" priority="49" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="170" priority="49" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G180))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="50">
@@ -14841,7 +14881,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G181:H181">
-    <cfRule type="containsText" dxfId="164" priority="47" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="169" priority="47" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G181))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="48">
@@ -14856,7 +14896,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G182:H182">
-    <cfRule type="containsText" dxfId="163" priority="43" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="168" priority="43" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G182))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="44">
@@ -14871,7 +14911,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G183:H183">
-    <cfRule type="containsText" dxfId="162" priority="41" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="167" priority="41" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G183))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="42">
@@ -14886,7 +14926,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G184:H184">
-    <cfRule type="containsText" dxfId="161" priority="39" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="166" priority="39" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G184))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="40">
@@ -14901,7 +14941,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G186:H186">
-    <cfRule type="containsText" dxfId="160" priority="35" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="165" priority="35" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G186))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="36">
@@ -14916,7 +14956,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G187:H187">
-    <cfRule type="containsText" dxfId="159" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="164" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G187))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -14931,7 +14971,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G188:H188">
-    <cfRule type="containsText" dxfId="158" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="163" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G188))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -14946,7 +14986,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G185:H185">
-    <cfRule type="containsText" dxfId="157" priority="29" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="162" priority="29" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G185))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="30">
@@ -14961,7 +15001,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G189:H189">
-    <cfRule type="containsText" dxfId="156" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="161" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G189))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -14976,7 +15016,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G190:H190">
-    <cfRule type="containsText" dxfId="155" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="160" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G190))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -14991,7 +15031,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G191:H191">
-    <cfRule type="containsText" dxfId="154" priority="23" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="159" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G191))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -15006,7 +15046,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H109">
-    <cfRule type="containsText" dxfId="153" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="158" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H109))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15023,7 +15063,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:H3">
-    <cfRule type="containsText" dxfId="152" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="157" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -15038,7 +15078,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G192">
-    <cfRule type="containsText" dxfId="151" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="156" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G192))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -15053,7 +15093,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H192">
-    <cfRule type="containsText" dxfId="150" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="155" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H192))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -15068,7 +15108,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G193:H193 G195:H195 G197:H197">
-    <cfRule type="containsText" dxfId="149" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="154" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G193))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -15083,7 +15123,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G194:H194 G196:H196">
-    <cfRule type="containsText" dxfId="148" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="153" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G194))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -15097,8 +15137,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G198 G200">
-    <cfRule type="containsText" dxfId="147" priority="9" operator="containsText" text="*-">
+  <conditionalFormatting sqref="G200 G198">
+    <cfRule type="containsText" dxfId="152" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G198))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -15112,8 +15152,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H198 H200">
-    <cfRule type="containsText" dxfId="146" priority="7" operator="containsText" text="*-">
+  <conditionalFormatting sqref="H200 H198">
+    <cfRule type="containsText" dxfId="151" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H198))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -15128,7 +15168,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G199:H199 G201:H201">
-    <cfRule type="containsText" dxfId="145" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="150" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G199))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -15143,7 +15183,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G202:H202">
-    <cfRule type="containsText" dxfId="144" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="149" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G202))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -15158,7 +15198,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G203:H203">
-    <cfRule type="containsText" dxfId="143" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="148" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G203))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -15949,8 +15989,8 @@
       <c r="F27" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G27" s="11" t="s">
-        <v>0</v>
+      <c r="G27" s="52">
+        <v>1</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>0</v>
@@ -16007,8 +16047,8 @@
       <c r="F29" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G29" s="11" t="s">
-        <v>0</v>
+      <c r="G29" s="52">
+        <v>1</v>
       </c>
       <c r="H29" s="11" t="s">
         <v>0</v>
@@ -16169,8 +16209,8 @@
       <c r="F35" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G35" s="11" t="s">
-        <v>0</v>
+      <c r="G35" s="52">
+        <v>1</v>
       </c>
       <c r="H35" s="11" t="s">
         <v>0</v>
@@ -16427,8 +16467,8 @@
       <c r="F44" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G44" s="11" t="s">
-        <v>0</v>
+      <c r="G44" s="52">
+        <v>1</v>
       </c>
       <c r="H44" s="11" t="s">
         <v>0</v>
@@ -16485,8 +16525,8 @@
       <c r="F46" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="G46" s="11" t="s">
-        <v>0</v>
+      <c r="G46" s="52">
+        <v>1</v>
       </c>
       <c r="H46" s="11" t="s">
         <v>0</v>
@@ -17899,10 +17939,10 @@
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <conditionalFormatting sqref="G15:H15 G17:H17 G26:H26 G19:H20 G22:H24">
-    <cfRule type="containsText" dxfId="142" priority="448" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="147" priority="458" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G15))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="449">
+    <cfRule type="colorScale" priority="459">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -17914,12 +17954,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="containsText" dxfId="141" priority="429" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="146" priority="439" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H26))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26">
-    <cfRule type="colorScale" priority="430">
+    <cfRule type="colorScale" priority="440">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -17931,10 +17971,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G28:H28">
-    <cfRule type="containsText" dxfId="140" priority="427" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="145" priority="437" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G28))))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="428">
+    <cfRule type="colorScale" priority="438">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -17946,11 +17986,58 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
-    <cfRule type="containsText" dxfId="139" priority="425" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="144" priority="435" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H28))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H28">
+    <cfRule type="colorScale" priority="436">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="containsText" dxfId="143" priority="433" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="434">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="containsText" dxfId="142" priority="431" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="colorScale" priority="432">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G32:H32">
+    <cfRule type="containsText" dxfId="141" priority="425" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="426">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -17962,10 +18049,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="138" priority="423" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H32">
+    <cfRule type="containsText" dxfId="140" priority="423" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H32))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32">
     <cfRule type="colorScale" priority="424">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -17977,12 +18066,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="137" priority="421" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
+  <conditionalFormatting sqref="G34:H34 G38:H38">
+    <cfRule type="containsText" dxfId="139" priority="421" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G34))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="422">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -17994,10 +18081,44 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G32:H32">
+  <conditionalFormatting sqref="H34 H38">
+    <cfRule type="containsText" dxfId="138" priority="419" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H34))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H34 H38">
+    <cfRule type="colorScale" priority="420">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G33:H33 G36:H36 G40:H40">
+    <cfRule type="containsText" dxfId="137" priority="417" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G33))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="418">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H33 H36 H40">
     <cfRule type="containsText" dxfId="136" priority="415" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G32))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H33 H36 H40">
     <cfRule type="colorScale" priority="416">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18009,12 +18130,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H32">
+  <conditionalFormatting sqref="G42:H42">
     <cfRule type="containsText" dxfId="135" priority="413" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H32))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H32">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G42))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="414">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18026,10 +18145,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G34:H34 G38:H38">
+  <conditionalFormatting sqref="H42">
     <cfRule type="containsText" dxfId="134" priority="411" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G34))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H42))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H42">
     <cfRule type="colorScale" priority="412">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18041,12 +18162,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H34 H38">
+  <conditionalFormatting sqref="G43:H43">
     <cfRule type="containsText" dxfId="133" priority="409" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H34))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H38 H34">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G43))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="410">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18058,10 +18177,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G33:H33 G36:H36 G40:H40">
+  <conditionalFormatting sqref="H43">
     <cfRule type="containsText" dxfId="132" priority="407" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G33))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H43))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H43">
     <cfRule type="colorScale" priority="408">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18073,12 +18194,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H33 H36 H40">
+  <conditionalFormatting sqref="G45:H45">
     <cfRule type="containsText" dxfId="131" priority="405" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H33))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H36 H33 H40">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G45))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="406">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18090,10 +18209,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G42:H42">
+  <conditionalFormatting sqref="H45">
     <cfRule type="containsText" dxfId="130" priority="403" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G42))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H45))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45">
     <cfRule type="colorScale" priority="404">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18105,12 +18226,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H42">
+  <conditionalFormatting sqref="G47:H47 G49:H49 G51:H51 G53:H53 G55:H56 G54">
     <cfRule type="containsText" dxfId="129" priority="401" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H42))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H42">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G47))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="402">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18122,10 +18241,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G43:H43">
+  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
     <cfRule type="containsText" dxfId="128" priority="399" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G43))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H47))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H49 H47 H51 H53 H55:H56">
     <cfRule type="colorScale" priority="400">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18137,12 +18258,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H43">
+  <conditionalFormatting sqref="G48:H48 G50:H50 G52:H52 H54">
     <cfRule type="containsText" dxfId="127" priority="397" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H43))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H43">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G48))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="398">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18154,10 +18273,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G45:H45">
+  <conditionalFormatting sqref="H48 H50 H52 H54">
     <cfRule type="containsText" dxfId="126" priority="395" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G45))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H48))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H48 H50 H52 H54">
     <cfRule type="colorScale" priority="396">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18169,13 +18290,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H45">
-    <cfRule type="containsText" dxfId="125" priority="393" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H45))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45">
-    <cfRule type="colorScale" priority="394">
+  <conditionalFormatting sqref="G61:H61 G63:H63 G65:H65 G67:H67 G69:H69">
+    <cfRule type="containsText" dxfId="125" priority="373" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G61))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="374">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18186,11 +18305,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G47:H47 G49:H49 G51:H51 G53:H53 G55:H56 G54">
-    <cfRule type="containsText" dxfId="124" priority="391" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G47))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="392">
+  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
+    <cfRule type="containsText" dxfId="124" priority="371" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H61))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H63 H61 H65 H67 H69">
+    <cfRule type="colorScale" priority="372">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18201,13 +18322,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
-    <cfRule type="containsText" dxfId="123" priority="389" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H47))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H47 H49 H51 H53 H55:H56">
-    <cfRule type="colorScale" priority="390">
+  <conditionalFormatting sqref="G60:H60 G62:H62 G64:H64 G66:H66 G68:H68 G70:H70 G73:H73">
+    <cfRule type="containsText" dxfId="123" priority="369" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G60))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="370">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18218,11 +18337,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G48:H48 G50:H50 G52:H52 H54">
-    <cfRule type="containsText" dxfId="122" priority="387" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G48))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="388">
+  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
+    <cfRule type="containsText" dxfId="122" priority="367" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H60))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H62 H60 H64 H66 H68 H70 H73">
+    <cfRule type="colorScale" priority="368">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18233,13 +18354,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H48 H50 H52 H54">
-    <cfRule type="containsText" dxfId="121" priority="385" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H48))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H50 H48 H52 H54">
-    <cfRule type="colorScale" priority="386">
+  <conditionalFormatting sqref="G58:H58">
+    <cfRule type="containsText" dxfId="121" priority="365" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G58))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="366">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18250,10 +18369,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G61:H61 G63:H63 G65:H65 G67:H67 G69:H69">
+  <conditionalFormatting sqref="H58">
     <cfRule type="containsText" dxfId="120" priority="363" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G61))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H58))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H58">
     <cfRule type="colorScale" priority="364">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18265,12 +18386,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
+  <conditionalFormatting sqref="G71:H71">
     <cfRule type="containsText" dxfId="119" priority="361" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H61))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H61 H63 H65 H67 H69">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G71))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="362">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18282,10 +18401,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G60:H60 G62:H62 G64:H64 G66:H66 G68:H68 G70:H70 G73:H73">
+  <conditionalFormatting sqref="H71">
     <cfRule type="containsText" dxfId="118" priority="359" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G60))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H71))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H71">
     <cfRule type="colorScale" priority="360">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18297,13 +18418,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
-    <cfRule type="containsText" dxfId="117" priority="357" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H60))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H60 H62 H64 H66 H68 H70 H73">
-    <cfRule type="colorScale" priority="358">
+  <conditionalFormatting sqref="G22">
+    <cfRule type="containsText" dxfId="117" priority="345" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G22))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="346">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18314,11 +18433,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G58:H58">
-    <cfRule type="containsText" dxfId="116" priority="355" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G58))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="356">
+  <conditionalFormatting sqref="H22">
+    <cfRule type="containsText" dxfId="116" priority="343" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H22))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="344">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18329,13 +18448,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H58">
-    <cfRule type="containsText" dxfId="115" priority="353" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H58))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H58">
-    <cfRule type="colorScale" priority="354">
+  <conditionalFormatting sqref="G25">
+    <cfRule type="containsText" dxfId="115" priority="341" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G25))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="342">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18346,56 +18463,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G71:H71">
-    <cfRule type="containsText" dxfId="114" priority="351" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G71))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="352">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H71">
-    <cfRule type="containsText" dxfId="113" priority="349" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H71))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H71">
-    <cfRule type="colorScale" priority="350">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G22">
-    <cfRule type="containsText" dxfId="112" priority="335" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G22))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="336">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H22">
-    <cfRule type="containsText" dxfId="111" priority="333" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H22))))</formula>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="containsText" dxfId="114" priority="333" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H27))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="334">
       <colorScale>
@@ -18408,10 +18478,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G25">
-    <cfRule type="containsText" dxfId="110" priority="331" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G25))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="containsText" dxfId="113" priority="331" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H27))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
     <cfRule type="colorScale" priority="332">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18423,11 +18495,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G27:H27">
-    <cfRule type="containsText" dxfId="109" priority="323" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="324">
+  <conditionalFormatting sqref="G75:H75">
+    <cfRule type="containsText" dxfId="112" priority="281" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G75))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="282">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18438,13 +18510,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="containsText" dxfId="108" priority="321" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H27))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="colorScale" priority="322">
+  <conditionalFormatting sqref="H75">
+    <cfRule type="containsText" dxfId="111" priority="279" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H75))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H75">
+    <cfRule type="colorScale" priority="280">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18455,10 +18527,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G75:H75">
-    <cfRule type="containsText" dxfId="107" priority="271" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G75))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="G77:H77">
+    <cfRule type="containsText" dxfId="110" priority="273" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G77))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="274">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H77">
+    <cfRule type="containsText" dxfId="109" priority="271" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H77))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H77">
     <cfRule type="colorScale" priority="272">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18470,13 +18559,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H75">
-    <cfRule type="containsText" dxfId="106" priority="269" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H75))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H75">
-    <cfRule type="colorScale" priority="270">
+  <conditionalFormatting sqref="G79:H79">
+    <cfRule type="containsText" dxfId="108" priority="265" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G79))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="266">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18487,10 +18574,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G77:H77">
-    <cfRule type="containsText" dxfId="105" priority="263" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G77))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H79">
+    <cfRule type="containsText" dxfId="107" priority="263" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H79))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H79">
     <cfRule type="colorScale" priority="264">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18502,12 +18591,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H77">
-    <cfRule type="containsText" dxfId="104" priority="261" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H77))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H77">
+  <conditionalFormatting sqref="G81:H81">
+    <cfRule type="containsText" dxfId="106" priority="261" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G81))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="262">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18519,10 +18606,44 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G79:H79">
+  <conditionalFormatting sqref="H81">
+    <cfRule type="containsText" dxfId="105" priority="259" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H81))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H81">
+    <cfRule type="colorScale" priority="260">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G83:H83">
+    <cfRule type="containsText" dxfId="104" priority="257" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G83))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="258">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H83">
     <cfRule type="containsText" dxfId="103" priority="255" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G79))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H83))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H83">
     <cfRule type="colorScale" priority="256">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18534,12 +18655,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H79">
+  <conditionalFormatting sqref="G85:H85">
     <cfRule type="containsText" dxfId="102" priority="253" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H79))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H79">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G85))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="254">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18551,10 +18670,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G81:H81">
+  <conditionalFormatting sqref="H85">
     <cfRule type="containsText" dxfId="101" priority="251" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G81))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H85))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H85">
     <cfRule type="colorScale" priority="252">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18566,13 +18687,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="containsText" dxfId="100" priority="249" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H81))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="colorScale" priority="250">
+  <conditionalFormatting sqref="H29">
+    <cfRule type="containsText" dxfId="99" priority="231" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="232">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18583,11 +18702,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G83:H83">
-    <cfRule type="containsText" dxfId="99" priority="247" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G83))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="248">
+  <conditionalFormatting sqref="H29">
+    <cfRule type="containsText" dxfId="98" priority="229" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29">
+    <cfRule type="colorScale" priority="230">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18598,13 +18719,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H83">
-    <cfRule type="containsText" dxfId="98" priority="245" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H83))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H83">
-    <cfRule type="colorScale" priority="246">
+  <conditionalFormatting sqref="H35">
+    <cfRule type="containsText" dxfId="96" priority="225" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="226">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18615,44 +18734,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G85:H85">
-    <cfRule type="containsText" dxfId="97" priority="243" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G85))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="244">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H85">
-    <cfRule type="containsText" dxfId="96" priority="241" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H85))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H85">
-    <cfRule type="colorScale" priority="242">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
+  <conditionalFormatting sqref="H35">
     <cfRule type="containsText" dxfId="95" priority="223" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
     <cfRule type="colorScale" priority="224">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18664,27 +18751,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G29:H29">
-    <cfRule type="containsText" dxfId="94" priority="221" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="222">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
+  <conditionalFormatting sqref="H44">
     <cfRule type="containsText" dxfId="93" priority="219" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H44))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="220">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18696,12 +18766,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
+  <conditionalFormatting sqref="H44">
     <cfRule type="containsText" dxfId="92" priority="217" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H44))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H44">
     <cfRule type="colorScale" priority="218">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18713,27 +18783,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G35:H35">
-    <cfRule type="containsText" dxfId="91" priority="215" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="216">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H35">
+  <conditionalFormatting sqref="H46">
     <cfRule type="containsText" dxfId="90" priority="213" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H35))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H35">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="214">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18745,12 +18798,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
+  <conditionalFormatting sqref="H46">
     <cfRule type="containsText" dxfId="89" priority="211" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H46">
     <cfRule type="colorScale" priority="212">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18762,27 +18815,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G44:H44">
-    <cfRule type="containsText" dxfId="88" priority="209" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="210">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H44">
-    <cfRule type="containsText" dxfId="87" priority="207" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H44))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H44">
+  <conditionalFormatting sqref="H59">
+    <cfRule type="containsText" dxfId="88" priority="207" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="208">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18794,12 +18830,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G44">
-    <cfRule type="containsText" dxfId="86" priority="205" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G44">
+  <conditionalFormatting sqref="H59">
+    <cfRule type="containsText" dxfId="87" priority="205" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H59">
     <cfRule type="colorScale" priority="206">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18811,27 +18847,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
-    <cfRule type="containsText" dxfId="85" priority="203" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="204">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
-    <cfRule type="containsText" dxfId="84" priority="201" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H46))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
+  <conditionalFormatting sqref="H57">
+    <cfRule type="containsText" dxfId="86" priority="201" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="202">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18843,11 +18862,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H59">
-    <cfRule type="containsText" dxfId="83" priority="197" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="198">
+  <conditionalFormatting sqref="H57">
+    <cfRule type="containsText" dxfId="85" priority="199" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H57">
+    <cfRule type="colorScale" priority="200">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18858,12 +18879,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H59">
-    <cfRule type="containsText" dxfId="82" priority="195" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H59))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H59">
+  <conditionalFormatting sqref="H80">
+    <cfRule type="containsText" dxfId="84" priority="195" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="196">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18875,11 +18894,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H57">
-    <cfRule type="containsText" dxfId="81" priority="191" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="192">
+  <conditionalFormatting sqref="H80">
+    <cfRule type="containsText" dxfId="83" priority="193" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H80">
+    <cfRule type="colorScale" priority="194">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18890,12 +18911,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H57">
-    <cfRule type="containsText" dxfId="80" priority="189" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H57))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H57">
+  <conditionalFormatting sqref="H78">
+    <cfRule type="containsText" dxfId="82" priority="189" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="190">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18907,11 +18926,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H80">
-    <cfRule type="containsText" dxfId="79" priority="185" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="186">
+  <conditionalFormatting sqref="H78">
+    <cfRule type="containsText" dxfId="81" priority="187" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H78">
+    <cfRule type="colorScale" priority="188">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18922,12 +18943,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H80">
-    <cfRule type="containsText" dxfId="78" priority="183" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H80))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H80">
+  <conditionalFormatting sqref="H76">
+    <cfRule type="containsText" dxfId="80" priority="183" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="184">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18939,11 +18958,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H78">
-    <cfRule type="containsText" dxfId="77" priority="179" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="180">
+  <conditionalFormatting sqref="H76">
+    <cfRule type="containsText" dxfId="79" priority="181" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H76">
+    <cfRule type="colorScale" priority="182">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18954,12 +18975,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H78">
-    <cfRule type="containsText" dxfId="76" priority="177" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H78))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H78">
+  <conditionalFormatting sqref="H74">
+    <cfRule type="containsText" dxfId="78" priority="177" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="178">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -18971,11 +18990,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H76">
-    <cfRule type="containsText" dxfId="75" priority="173" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="174">
+  <conditionalFormatting sqref="H74">
+    <cfRule type="containsText" dxfId="77" priority="175" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H74">
+    <cfRule type="colorScale" priority="176">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -18986,12 +19007,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H76">
-    <cfRule type="containsText" dxfId="74" priority="171" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H76))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H76">
+  <conditionalFormatting sqref="H72">
+    <cfRule type="containsText" dxfId="76" priority="171" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="172">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19003,11 +19022,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H74">
-    <cfRule type="containsText" dxfId="73" priority="167" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="168">
+  <conditionalFormatting sqref="H72">
+    <cfRule type="containsText" dxfId="75" priority="169" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H72">
+    <cfRule type="colorScale" priority="170">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19018,12 +19039,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H74">
-    <cfRule type="containsText" dxfId="72" priority="165" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H74))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H74">
+  <conditionalFormatting sqref="H82">
+    <cfRule type="containsText" dxfId="74" priority="165" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="166">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19035,11 +19054,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H72">
-    <cfRule type="containsText" dxfId="71" priority="161" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="162">
+  <conditionalFormatting sqref="H82">
+    <cfRule type="containsText" dxfId="73" priority="163" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H82">
+    <cfRule type="colorScale" priority="164">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19050,12 +19071,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H72">
-    <cfRule type="containsText" dxfId="70" priority="159" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H72))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H72">
+  <conditionalFormatting sqref="H86">
+    <cfRule type="containsText" dxfId="72" priority="159" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="160">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19067,11 +19086,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H82">
-    <cfRule type="containsText" dxfId="69" priority="155" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="156">
+  <conditionalFormatting sqref="H86">
+    <cfRule type="containsText" dxfId="71" priority="157" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H86">
+    <cfRule type="colorScale" priority="158">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19082,12 +19103,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H82">
-    <cfRule type="containsText" dxfId="68" priority="153" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H82))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H82">
+  <conditionalFormatting sqref="H84">
+    <cfRule type="containsText" dxfId="70" priority="153" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="154">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19099,11 +19118,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
-    <cfRule type="containsText" dxfId="67" priority="149" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="150">
+  <conditionalFormatting sqref="H84">
+    <cfRule type="containsText" dxfId="69" priority="151" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H84">
+    <cfRule type="colorScale" priority="152">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19114,12 +19135,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
-    <cfRule type="containsText" dxfId="66" priority="147" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H86))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H86">
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="68" priority="147" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="148">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19131,11 +19150,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H84">
-    <cfRule type="containsText" dxfId="65" priority="143" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="144">
+  <conditionalFormatting sqref="H37">
+    <cfRule type="containsText" dxfId="67" priority="145" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="colorScale" priority="146">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19146,12 +19167,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H84">
-    <cfRule type="containsText" dxfId="64" priority="141" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H84))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H84">
+  <conditionalFormatting sqref="H41">
+    <cfRule type="containsText" dxfId="66" priority="141" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="142">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19163,11 +19182,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
-    <cfRule type="containsText" dxfId="63" priority="137" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="138">
+  <conditionalFormatting sqref="H41">
+    <cfRule type="containsText" dxfId="65" priority="139" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H41">
+    <cfRule type="colorScale" priority="140">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19178,12 +19199,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
-    <cfRule type="containsText" dxfId="62" priority="135" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H37))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
+  <conditionalFormatting sqref="H39">
+    <cfRule type="containsText" dxfId="64" priority="135" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="136">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19195,11 +19214,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H41">
-    <cfRule type="containsText" dxfId="61" priority="131" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="132">
+  <conditionalFormatting sqref="H39">
+    <cfRule type="containsText" dxfId="63" priority="133" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H39">
+    <cfRule type="colorScale" priority="134">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19210,13 +19231,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H41">
-    <cfRule type="containsText" dxfId="60" priority="129" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H41))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H41">
-    <cfRule type="colorScale" priority="130">
+  <conditionalFormatting sqref="G21">
+    <cfRule type="containsText" dxfId="62" priority="127" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G21))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="128">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19227,27 +19246,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H39">
-    <cfRule type="containsText" dxfId="59" priority="125" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="126">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H39">
-    <cfRule type="containsText" dxfId="58" priority="123" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H39))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H39">
+  <conditionalFormatting sqref="G18">
+    <cfRule type="containsText" dxfId="61" priority="123" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="124">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19259,11 +19261,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G21">
-    <cfRule type="containsText" dxfId="57" priority="117" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G21))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="118">
+  <conditionalFormatting sqref="G16">
+    <cfRule type="containsText" dxfId="60" priority="119" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G16))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="120">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19274,9 +19276,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G18">
-    <cfRule type="containsText" dxfId="56" priority="113" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G18))))</formula>
+  <conditionalFormatting sqref="H31">
+    <cfRule type="containsText" dxfId="59" priority="113" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="114">
       <colorScale>
@@ -19289,11 +19291,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16">
-    <cfRule type="containsText" dxfId="55" priority="109" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G16))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="110">
+  <conditionalFormatting sqref="H31">
+    <cfRule type="containsText" dxfId="58" priority="111" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H31">
+    <cfRule type="colorScale" priority="112">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19304,9 +19308,39 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
-    <cfRule type="containsText" dxfId="54" priority="103" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
+  <conditionalFormatting sqref="G3:H8">
+    <cfRule type="containsText" dxfId="57" priority="107" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="108">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:G14">
+    <cfRule type="containsText" dxfId="56" priority="105" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G9))))</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="106">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:H14">
+    <cfRule type="containsText" dxfId="55" priority="103" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="104">
       <colorScale>
@@ -19319,12 +19353,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
-    <cfRule type="containsText" dxfId="53" priority="101" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H31))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
+  <conditionalFormatting sqref="G87:H87">
+    <cfRule type="containsText" dxfId="54" priority="101" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G87))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="102">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19336,9 +19368,26 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:H8">
+  <conditionalFormatting sqref="H87">
+    <cfRule type="containsText" dxfId="53" priority="99" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H87))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H87">
+    <cfRule type="colorScale" priority="100">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H88">
     <cfRule type="containsText" dxfId="52" priority="97" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="98">
       <colorScale>
@@ -19351,10 +19400,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:G14">
+  <conditionalFormatting sqref="H88">
     <cfRule type="containsText" dxfId="51" priority="95" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G9))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H88">
     <cfRule type="colorScale" priority="96">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19366,24 +19417,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H14">
-    <cfRule type="containsText" dxfId="50" priority="93" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H9))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="94">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G87:H87">
-    <cfRule type="containsText" dxfId="49" priority="91" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G87))))</formula>
+  <conditionalFormatting sqref="G31">
+    <cfRule type="containsText" dxfId="50" priority="91" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G31))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="92">
       <colorScale>
@@ -19396,12 +19432,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H87">
-    <cfRule type="containsText" dxfId="48" priority="89" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H87))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H87">
+  <conditionalFormatting sqref="G89:H89">
+    <cfRule type="containsText" dxfId="49" priority="89" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G89))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="90">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19413,10 +19447,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="47" priority="87" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="H89">
+    <cfRule type="containsText" dxfId="48" priority="87" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H89))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H89">
     <cfRule type="colorScale" priority="88">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19428,12 +19464,10 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
-    <cfRule type="containsText" dxfId="46" priority="85" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H88))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H88">
+  <conditionalFormatting sqref="H90">
+    <cfRule type="containsText" dxfId="47" priority="85" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19445,11 +19479,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G31">
-    <cfRule type="containsText" dxfId="45" priority="81" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G31))))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="82">
+  <conditionalFormatting sqref="H90">
+    <cfRule type="containsText" dxfId="46" priority="83" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H90">
+    <cfRule type="colorScale" priority="84">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19460,9 +19496,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G89:H89">
-    <cfRule type="containsText" dxfId="44" priority="79" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G89))))</formula>
+  <conditionalFormatting sqref="H91:H94">
+    <cfRule type="containsText" dxfId="45" priority="79" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="80">
       <colorScale>
@@ -19475,12 +19511,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H89">
-    <cfRule type="containsText" dxfId="43" priority="77" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H89))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H89">
+  <conditionalFormatting sqref="H91:H94">
+    <cfRule type="containsText" dxfId="44" priority="77" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H91:H94">
     <cfRule type="colorScale" priority="78">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19492,9 +19528,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H90">
-    <cfRule type="containsText" dxfId="42" priority="75" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
+  <conditionalFormatting sqref="H95">
+    <cfRule type="containsText" dxfId="43" priority="75" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="76">
       <colorScale>
@@ -19507,12 +19543,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H90">
-    <cfRule type="containsText" dxfId="41" priority="73" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H90))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H90">
+  <conditionalFormatting sqref="H95">
+    <cfRule type="containsText" dxfId="42" priority="73" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H95">
     <cfRule type="colorScale" priority="74">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19524,10 +19560,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H91:H94">
-    <cfRule type="containsText" dxfId="40" priority="69" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="G30">
+    <cfRule type="containsText" dxfId="41" priority="69" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G30))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30">
     <cfRule type="colorScale" priority="70">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19539,12 +19577,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H91:H94">
-    <cfRule type="containsText" dxfId="39" priority="67" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H91))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H91:H94">
+  <conditionalFormatting sqref="G91">
+    <cfRule type="containsText" dxfId="40" priority="67" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G91))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G91">
     <cfRule type="colorScale" priority="68">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19556,10 +19594,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H95">
-    <cfRule type="containsText" dxfId="38" priority="65" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
-    </cfRule>
+  <conditionalFormatting sqref="G92">
+    <cfRule type="containsText" dxfId="39" priority="65" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G92))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G92">
     <cfRule type="colorScale" priority="66">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19571,12 +19611,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H95">
-    <cfRule type="containsText" dxfId="37" priority="63" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H95))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H95">
+  <conditionalFormatting sqref="G93">
+    <cfRule type="containsText" dxfId="38" priority="63" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G93))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G93">
     <cfRule type="colorScale" priority="64">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19588,12 +19628,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
-    <cfRule type="containsText" dxfId="36" priority="59" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G30))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
+  <conditionalFormatting sqref="G94">
+    <cfRule type="containsText" dxfId="37" priority="59" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G94))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G94">
     <cfRule type="colorScale" priority="60">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19605,12 +19645,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G91">
-    <cfRule type="containsText" dxfId="35" priority="57" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G91))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G91">
+  <conditionalFormatting sqref="G95">
+    <cfRule type="containsText" dxfId="36" priority="57" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G95))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G95">
     <cfRule type="colorScale" priority="58">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19622,12 +19662,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G92">
-    <cfRule type="containsText" dxfId="34" priority="55" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G92))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G92">
+  <conditionalFormatting sqref="G90">
+    <cfRule type="containsText" dxfId="35" priority="55" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G90))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G90">
     <cfRule type="colorScale" priority="56">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19639,13 +19679,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G93">
-    <cfRule type="containsText" dxfId="33" priority="53" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G93))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G93">
-    <cfRule type="colorScale" priority="54">
+  <conditionalFormatting sqref="G59">
+    <cfRule type="containsText" dxfId="34" priority="51" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G59))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G59">
+    <cfRule type="colorScale" priority="52">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19656,12 +19696,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G94">
-    <cfRule type="containsText" dxfId="32" priority="49" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G94))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G94">
+  <conditionalFormatting sqref="G76">
+    <cfRule type="containsText" dxfId="33" priority="49" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G76))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G76">
     <cfRule type="colorScale" priority="50">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19673,29 +19713,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G95">
-    <cfRule type="containsText" dxfId="31" priority="47" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G95))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G95">
-    <cfRule type="colorScale" priority="48">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G90">
-    <cfRule type="containsText" dxfId="30" priority="45" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G90))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G90">
+  <conditionalFormatting sqref="G80">
+    <cfRule type="containsText" dxfId="32" priority="45" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G80))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G80">
     <cfRule type="colorScale" priority="46">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19707,12 +19730,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G59">
-    <cfRule type="containsText" dxfId="29" priority="41" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G59))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G59">
+  <conditionalFormatting sqref="G82">
+    <cfRule type="containsText" dxfId="31" priority="43" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G82))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G82">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G84">
+    <cfRule type="containsText" dxfId="30" priority="41" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G84))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G84">
     <cfRule type="colorScale" priority="42">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19724,12 +19764,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G76">
-    <cfRule type="containsText" dxfId="28" priority="39" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G76))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G76">
+  <conditionalFormatting sqref="G88">
+    <cfRule type="containsText" dxfId="29" priority="39" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G88))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G88">
     <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19741,13 +19781,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G80">
-    <cfRule type="containsText" dxfId="27" priority="35" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G80))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G80">
-    <cfRule type="colorScale" priority="36">
+  <conditionalFormatting sqref="G86">
+    <cfRule type="containsText" dxfId="28" priority="37" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G86))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G86">
+    <cfRule type="colorScale" priority="38">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -19758,29 +19798,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G82">
-    <cfRule type="containsText" dxfId="26" priority="33" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G82))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G82">
-    <cfRule type="colorScale" priority="34">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G84">
+  <conditionalFormatting sqref="G74">
     <cfRule type="containsText" dxfId="25" priority="31" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G84))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G84">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G74))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G74">
     <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19792,12 +19815,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G88">
+  <conditionalFormatting sqref="G57">
     <cfRule type="containsText" dxfId="24" priority="29" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G88))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G88">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G57))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G57">
     <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19809,12 +19832,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G86">
+  <conditionalFormatting sqref="G78">
     <cfRule type="containsText" dxfId="23" priority="27" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G86))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G86">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G78))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G78">
     <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19826,10 +19849,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
+  <conditionalFormatting sqref="H16">
     <cfRule type="containsText" dxfId="22" priority="25" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
-    </cfRule>
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
     <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19841,12 +19866,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
+  <conditionalFormatting sqref="H18">
     <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H18))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
     <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19858,12 +19883,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G74">
+  <conditionalFormatting sqref="H21">
     <cfRule type="containsText" dxfId="20" priority="21" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G74))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G74">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H21))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H21">
     <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19875,12 +19900,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G57">
+  <conditionalFormatting sqref="H25">
     <cfRule type="containsText" dxfId="19" priority="19" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G57))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H25))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19892,12 +19917,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G78">
+  <conditionalFormatting sqref="G41">
     <cfRule type="containsText" dxfId="18" priority="17" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G78))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G78">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G41))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G41">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19909,12 +19934,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H16">
+  <conditionalFormatting sqref="G39">
     <cfRule type="containsText" dxfId="17" priority="15" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H16">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G39))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G39">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19926,12 +19951,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H18">
+  <conditionalFormatting sqref="G37">
     <cfRule type="containsText" dxfId="16" priority="13" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H18))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H18">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G37))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19943,12 +19968,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
+  <conditionalFormatting sqref="G72">
     <cfRule type="containsText" dxfId="15" priority="11" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H21))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G72))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G72">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19960,12 +19985,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H25">
-    <cfRule type="containsText" dxfId="14" priority="9" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H25))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H25">
+  <conditionalFormatting sqref="G27">
+    <cfRule type="containsText" dxfId="4" priority="9" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G27))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19977,12 +20002,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G41">
-    <cfRule type="containsText" dxfId="13" priority="7" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G41))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G41">
+  <conditionalFormatting sqref="G29">
+    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -19994,12 +20019,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G39">
-    <cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G39))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G39">
+  <conditionalFormatting sqref="G35">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G35))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20011,12 +20036,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G37">
-    <cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G37))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G37">
+  <conditionalFormatting sqref="G44">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G44))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20028,12 +20053,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G72">
-    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(G72))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G72">
+  <conditionalFormatting sqref="G46">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(G46))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G46">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -20949,7 +20974,7 @@
     <mergeCell ref="G1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3:H28">
-    <cfRule type="containsText" dxfId="9" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="14" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -20964,7 +20989,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H29">
-    <cfRule type="containsText" dxfId="8" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="13" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -20979,7 +21004,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H29">
-    <cfRule type="containsText" dxfId="7" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H29))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20996,7 +21021,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G29">
-    <cfRule type="containsText" dxfId="6" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G29))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21013,7 +21038,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="5" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -21028,7 +21053,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H30">
-    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H30))))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21045,7 +21070,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(G30))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">

</xml_diff>